<commit_message>
ingesta: snapshot 2026-07-26 18:07 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-07-26/Temp-max-julio-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-07-26/Temp-max-julio-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.187.8\Oficina\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94541FB-387C-4BF0-BA2B-96323FE62BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7597456B-DDE2-4EBA-96A3-483CE8F848A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9496,7 +9496,9 @@
       <c r="AB5" s="57">
         <v>30.7</v>
       </c>
-      <c r="AC5" s="57"/>
+      <c r="AC5" s="57">
+        <v>30.8</v>
+      </c>
       <c r="AD5" s="57"/>
       <c r="AE5" s="57"/>
       <c r="AF5" s="57"/>
@@ -9505,7 +9507,7 @@
       <c r="AI5" s="57"/>
       <c r="AJ5" s="37">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>30.7</v>
+        <v>30.8</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9523,11 +9525,11 @@
       </c>
       <c r="AO5" s="23">
         <f>IF(COUNTIF(E5:AI5,"&gt;0")&gt;=15,AVERAGE(E5:AI5),"")</f>
-        <v>31.050000000000008</v>
+        <v>31.040000000000006</v>
       </c>
       <c r="AP5" s="23">
         <f>IF(AN5&gt;0,IFERROR(AO5-AN5,""),"")</f>
-        <v>0.85262822399177907</v>
+        <v>0.8426282239917775</v>
       </c>
     </row>
     <row r="6" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9615,7 +9617,9 @@
       <c r="AB6" s="57">
         <v>29.7</v>
       </c>
-      <c r="AC6" s="57"/>
+      <c r="AC6" s="57">
+        <v>30.6</v>
+      </c>
       <c r="AD6" s="57"/>
       <c r="AE6" s="57"/>
       <c r="AF6" s="57"/>
@@ -9624,7 +9628,7 @@
       <c r="AI6" s="57"/>
       <c r="AJ6" s="37">
         <f t="shared" ref="AJ6:AJ48" si="0">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>29.7</v>
+        <v>30.6</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="1">+MAX($E6:$AI6)</f>
@@ -9642,11 +9646,11 @@
       </c>
       <c r="AO6" s="23">
         <f t="shared" ref="AO6:AO15" si="3">IF(COUNTIF(E6:AI6,"&gt;0")&gt;=15,AVERAGE(E6:AI6),"")</f>
-        <v>30.612499999999997</v>
+        <v>30.611999999999998</v>
       </c>
       <c r="AP6" s="23">
         <f t="shared" ref="AP6:AP48" si="4">IF(AN6&gt;0,IFERROR(AO6-AN6,""),"")</f>
-        <v>-4.1780397022343152E-2</v>
+        <v>-4.2280397022341987E-2</v>
       </c>
     </row>
     <row r="7" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9734,7 +9738,9 @@
       <c r="AB7" s="57">
         <v>32.700000000000003</v>
       </c>
-      <c r="AC7" s="57"/>
+      <c r="AC7" s="57">
+        <v>36.6</v>
+      </c>
       <c r="AD7" s="57"/>
       <c r="AE7" s="57"/>
       <c r="AF7" s="57"/>
@@ -9743,7 +9749,7 @@
       <c r="AI7" s="57"/>
       <c r="AJ7" s="37">
         <f t="shared" si="0"/>
-        <v>32.700000000000003</v>
+        <v>36.6</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9761,11 +9767,11 @@
       </c>
       <c r="AO7" s="23">
         <f t="shared" si="3"/>
-        <v>35.420833333333334</v>
+        <v>35.468000000000004</v>
       </c>
       <c r="AP7" s="23">
         <f t="shared" si="4"/>
-        <v>2.0548173257642617</v>
+        <v>2.1019839924309309</v>
       </c>
     </row>
     <row r="8" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9853,7 +9859,9 @@
       <c r="AB8" s="57">
         <v>32.200000000000003</v>
       </c>
-      <c r="AC8" s="57"/>
+      <c r="AC8" s="57">
+        <v>33.4</v>
+      </c>
       <c r="AD8" s="57"/>
       <c r="AE8" s="57"/>
       <c r="AF8" s="57"/>
@@ -9862,7 +9870,7 @@
       <c r="AI8" s="57"/>
       <c r="AJ8" s="37">
         <f t="shared" si="0"/>
-        <v>32.200000000000003</v>
+        <v>33.4</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
@@ -9880,11 +9888,11 @@
       </c>
       <c r="AO8" s="23">
         <f t="shared" si="3"/>
-        <v>33.162500000000001</v>
+        <v>33.172000000000004</v>
       </c>
       <c r="AP8" s="23">
         <f t="shared" si="4"/>
-        <v>0.91345698924730812</v>
+        <v>0.92295698924731084</v>
       </c>
     </row>
     <row r="9" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9972,7 +9980,9 @@
       <c r="AB9" s="57">
         <v>34.1</v>
       </c>
-      <c r="AC9" s="57"/>
+      <c r="AC9" s="57">
+        <v>33.299999999999997</v>
+      </c>
       <c r="AD9" s="57"/>
       <c r="AE9" s="57"/>
       <c r="AF9" s="57"/>
@@ -9981,7 +9991,7 @@
       <c r="AI9" s="57"/>
       <c r="AJ9" s="37">
         <f t="shared" si="0"/>
-        <v>34.1</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -9999,11 +10009,11 @@
       </c>
       <c r="AO9" s="23">
         <f t="shared" si="3"/>
-        <v>33.791666666666664</v>
+        <v>33.771999999999998</v>
       </c>
       <c r="AP9" s="23">
         <f t="shared" si="4"/>
-        <v>0.70042052898281781</v>
+        <v>0.68075386231615198</v>
       </c>
     </row>
     <row r="10" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10091,7 +10101,9 @@
       <c r="AB10" s="57">
         <v>36.6</v>
       </c>
-      <c r="AC10" s="57"/>
+      <c r="AC10" s="57">
+        <v>36.299999999999997</v>
+      </c>
       <c r="AD10" s="57"/>
       <c r="AE10" s="57"/>
       <c r="AF10" s="57"/>
@@ -10100,7 +10112,7 @@
       <c r="AI10" s="57"/>
       <c r="AJ10" s="37">
         <f t="shared" si="0"/>
-        <v>36.6</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -10118,11 +10130,11 @@
       </c>
       <c r="AO10" s="23">
         <f t="shared" si="3"/>
-        <v>35.816666666666663</v>
+        <v>35.835999999999991</v>
       </c>
       <c r="AP10" s="23">
         <f t="shared" si="4"/>
-        <v>0.43642843900630623</v>
+        <v>0.45576177233963477</v>
       </c>
     </row>
     <row r="11" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10210,7 +10222,9 @@
       <c r="AB11" s="57">
         <v>38.799999999999997</v>
       </c>
-      <c r="AC11" s="57"/>
+      <c r="AC11" s="57">
+        <v>39.4</v>
+      </c>
       <c r="AD11" s="57"/>
       <c r="AE11" s="57"/>
       <c r="AF11" s="57"/>
@@ -10219,7 +10233,7 @@
       <c r="AI11" s="57"/>
       <c r="AJ11" s="37">
         <f t="shared" si="0"/>
-        <v>38.799999999999997</v>
+        <v>39.4</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -10237,11 +10251,11 @@
       </c>
       <c r="AO11" s="23">
         <f t="shared" si="3"/>
-        <v>37.983333333333327</v>
+        <v>38.039999999999992</v>
       </c>
       <c r="AP11" s="23">
         <f t="shared" si="4"/>
-        <v>2.4460492404847258</v>
+        <v>2.5027159071513907</v>
       </c>
     </row>
     <row r="12" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10329,7 +10343,9 @@
       <c r="AB12" s="57">
         <v>33.799999999999997</v>
       </c>
-      <c r="AC12" s="57"/>
+      <c r="AC12" s="57">
+        <v>33.799999999999997</v>
+      </c>
       <c r="AD12" s="57"/>
       <c r="AE12" s="57"/>
       <c r="AF12" s="57"/>
@@ -10356,11 +10372,11 @@
       </c>
       <c r="AO12" s="23">
         <f t="shared" si="3"/>
-        <v>34.708333333333329</v>
+        <v>34.671999999999997</v>
       </c>
       <c r="AP12" s="23">
         <f t="shared" si="4"/>
-        <v>2.5197091871595916</v>
+        <v>2.48337585382626</v>
       </c>
     </row>
     <row r="13" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10448,7 +10464,9 @@
       <c r="AB13" s="57">
         <v>34.4</v>
       </c>
-      <c r="AC13" s="57"/>
+      <c r="AC13" s="57">
+        <v>35.4</v>
+      </c>
       <c r="AD13" s="57"/>
       <c r="AE13" s="57"/>
       <c r="AF13" s="57"/>
@@ -10457,7 +10475,7 @@
       <c r="AI13" s="57"/>
       <c r="AJ13" s="37">
         <f t="shared" si="0"/>
-        <v>34.4</v>
+        <v>35.4</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10475,11 +10493,11 @@
       </c>
       <c r="AO13" s="23">
         <f t="shared" si="3"/>
-        <v>35.416666666666664</v>
+        <v>35.415999999999997</v>
       </c>
       <c r="AP13" s="23">
         <f t="shared" si="4"/>
-        <v>2.0348745519713276</v>
+        <v>2.0342078853046601</v>
       </c>
     </row>
     <row r="14" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10567,7 +10585,9 @@
       <c r="AB14" s="57">
         <v>34.4</v>
       </c>
-      <c r="AC14" s="57"/>
+      <c r="AC14" s="57">
+        <v>36</v>
+      </c>
       <c r="AD14" s="57"/>
       <c r="AE14" s="57"/>
       <c r="AF14" s="57"/>
@@ -10576,7 +10596,7 @@
       <c r="AI14" s="57"/>
       <c r="AJ14" s="37">
         <f t="shared" si="0"/>
-        <v>34.4</v>
+        <v>36</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
@@ -10594,11 +10614,11 @@
       </c>
       <c r="AO14" s="23">
         <f t="shared" si="3"/>
-        <v>34.68333333333333</v>
+        <v>34.735999999999997</v>
       </c>
       <c r="AP14" s="23">
         <f t="shared" si="4"/>
-        <v>1.4583967341190984</v>
+        <v>1.5110634007857655</v>
       </c>
     </row>
     <row r="15" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10686,7 +10706,9 @@
       <c r="AB15" s="57">
         <v>32.200000000000003</v>
       </c>
-      <c r="AC15" s="57"/>
+      <c r="AC15" s="57">
+        <v>33.4</v>
+      </c>
       <c r="AD15" s="57"/>
       <c r="AE15" s="57"/>
       <c r="AF15" s="57"/>
@@ -10695,7 +10717,7 @@
       <c r="AI15" s="57"/>
       <c r="AJ15" s="37">
         <f t="shared" si="0"/>
-        <v>32.200000000000003</v>
+        <v>33.4</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
@@ -10713,11 +10735,11 @@
       </c>
       <c r="AO15" s="23">
         <f t="shared" si="3"/>
-        <v>31.716666666666665</v>
+        <v>31.783999999999995</v>
       </c>
       <c r="AP15" s="23">
         <f t="shared" si="4"/>
-        <v>-1.8670789413285149E-2</v>
+        <v>4.8662543920045209E-2</v>
       </c>
     </row>
     <row r="16" spans="1:46" s="2" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -10854,7 +10876,9 @@
       <c r="AB17" s="57">
         <v>33.6</v>
       </c>
-      <c r="AC17" s="57"/>
+      <c r="AC17" s="57">
+        <v>35</v>
+      </c>
       <c r="AD17" s="57"/>
       <c r="AE17" s="57"/>
       <c r="AF17" s="57"/>
@@ -10863,7 +10887,7 @@
       <c r="AI17" s="57"/>
       <c r="AJ17" s="37">
         <f t="shared" si="0"/>
-        <v>33.6</v>
+        <v>35</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
@@ -10881,11 +10905,11 @@
       </c>
       <c r="AO17" s="23">
         <f>IF(COUNTIF(E17:AI17,"&gt;0")&gt;=15,AVERAGE(E17:AI17),"")</f>
-        <v>34.12083333333333</v>
+        <v>34.155999999999992</v>
       </c>
       <c r="AP17" s="23">
         <f>IF(AN17&gt;0,IFERROR(AO17-AN17,""),"")</f>
-        <v>1.4468511308861736</v>
+        <v>1.4820177975528352</v>
       </c>
     </row>
     <row r="18" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10973,7 +10997,9 @@
       <c r="AB18" s="57">
         <v>27.5</v>
       </c>
-      <c r="AC18" s="57"/>
+      <c r="AC18" s="57">
+        <v>28.2</v>
+      </c>
       <c r="AD18" s="57"/>
       <c r="AE18" s="57"/>
       <c r="AF18" s="57"/>
@@ -10982,7 +11008,7 @@
       <c r="AI18" s="57"/>
       <c r="AJ18" s="37">
         <f t="shared" si="0"/>
-        <v>27.5</v>
+        <v>28.2</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="1"/>
@@ -11000,11 +11026,11 @@
       </c>
       <c r="AO18" s="23">
         <f t="shared" ref="AO18:AO33" si="5">IF(COUNTIF(E18:AI18,"&gt;0")&gt;=15,AVERAGE(E18:AI18),"")</f>
-        <v>27.837500000000006</v>
+        <v>27.852000000000007</v>
       </c>
       <c r="AP18" s="23">
         <f t="shared" si="4"/>
-        <v>1.7776291460431359</v>
+        <v>1.7921291460431377</v>
       </c>
     </row>
     <row r="19" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11092,7 +11118,9 @@
       <c r="AB19" s="57">
         <v>35.299999999999997</v>
       </c>
-      <c r="AC19" s="57"/>
+      <c r="AC19" s="57">
+        <v>34</v>
+      </c>
       <c r="AD19" s="57"/>
       <c r="AE19" s="57"/>
       <c r="AF19" s="57"/>
@@ -11101,7 +11129,7 @@
       <c r="AI19" s="57"/>
       <c r="AJ19" s="37">
         <f t="shared" si="0"/>
-        <v>35.299999999999997</v>
+        <v>34</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="1"/>
@@ -11119,11 +11147,11 @@
       </c>
       <c r="AO19" s="23">
         <f t="shared" si="5"/>
-        <v>33.68333333333333</v>
+        <v>33.695999999999998</v>
       </c>
       <c r="AP19" s="23">
         <f t="shared" si="4"/>
-        <v>0.43237093066368715</v>
+        <v>0.44503759733035508</v>
       </c>
     </row>
     <row r="20" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11211,7 +11239,9 @@
       <c r="AB20" s="57">
         <v>30.3</v>
       </c>
-      <c r="AC20" s="57"/>
+      <c r="AC20" s="57">
+        <v>30.6</v>
+      </c>
       <c r="AD20" s="57"/>
       <c r="AE20" s="57"/>
       <c r="AF20" s="57"/>
@@ -11220,7 +11250,7 @@
       <c r="AI20" s="57"/>
       <c r="AJ20" s="37">
         <f t="shared" si="0"/>
-        <v>30.3</v>
+        <v>30.6</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="1"/>
@@ -11238,11 +11268,11 @@
       </c>
       <c r="AO20" s="23">
         <f t="shared" si="5"/>
-        <v>30.200000000000003</v>
+        <v>30.216000000000005</v>
       </c>
       <c r="AP20" s="23">
         <f t="shared" si="4"/>
-        <v>1.5591954022988546</v>
+        <v>1.5751954022988564</v>
       </c>
     </row>
     <row r="21" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11330,7 +11360,9 @@
       <c r="AB21" s="57">
         <v>23.5</v>
       </c>
-      <c r="AC21" s="57"/>
+      <c r="AC21" s="57">
+        <v>23.9</v>
+      </c>
       <c r="AD21" s="57"/>
       <c r="AE21" s="57"/>
       <c r="AF21" s="57"/>
@@ -11339,7 +11371,7 @@
       <c r="AI21" s="57"/>
       <c r="AJ21" s="37">
         <f t="shared" si="0"/>
-        <v>23.5</v>
+        <v>23.9</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -11357,11 +11389,11 @@
       </c>
       <c r="AO21" s="23">
         <f t="shared" si="5"/>
-        <v>24.266666666666662</v>
+        <v>24.251999999999995</v>
       </c>
       <c r="AP21" s="23">
         <f t="shared" si="4"/>
-        <v>1.6571635150166912</v>
+        <v>1.6424968483500244</v>
       </c>
     </row>
     <row r="22" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11517,7 +11549,9 @@
       <c r="AB23" s="57">
         <v>28.2</v>
       </c>
-      <c r="AC23" s="57"/>
+      <c r="AC23" s="57">
+        <v>28.8</v>
+      </c>
       <c r="AD23" s="57"/>
       <c r="AE23" s="57"/>
       <c r="AF23" s="57"/>
@@ -11526,7 +11560,7 @@
       <c r="AI23" s="57"/>
       <c r="AJ23" s="37">
         <f t="shared" si="0"/>
-        <v>28.2</v>
+        <v>28.8</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -11544,11 +11578,11 @@
       </c>
       <c r="AO23" s="23">
         <f t="shared" si="5"/>
-        <v>28.583333333333339</v>
+        <v>28.592000000000002</v>
       </c>
       <c r="AP23" s="23">
         <f t="shared" si="4"/>
-        <v>1.7149462365591397</v>
+        <v>1.7236129032258027</v>
       </c>
     </row>
     <row r="24" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11636,7 +11670,9 @@
       <c r="AB24" s="57">
         <v>29.6</v>
       </c>
-      <c r="AC24" s="57"/>
+      <c r="AC24" s="57">
+        <v>28.6</v>
+      </c>
       <c r="AD24" s="57"/>
       <c r="AE24" s="57"/>
       <c r="AF24" s="57"/>
@@ -11645,7 +11681,7 @@
       <c r="AI24" s="57"/>
       <c r="AJ24" s="37">
         <f t="shared" si="0"/>
-        <v>29.6</v>
+        <v>28.6</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="1"/>
@@ -11663,11 +11699,11 @@
       </c>
       <c r="AO24" s="23">
         <f t="shared" si="5"/>
-        <v>29.554166666666671</v>
+        <v>29.516000000000005</v>
       </c>
       <c r="AP24" s="23">
         <f t="shared" si="4"/>
-        <v>1.3023425499231891</v>
+        <v>1.2641758832565237</v>
       </c>
     </row>
     <row r="25" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11755,7 +11791,9 @@
       <c r="AB25" s="57">
         <v>33.700000000000003</v>
       </c>
-      <c r="AC25" s="57"/>
+      <c r="AC25" s="57">
+        <v>32.6</v>
+      </c>
       <c r="AD25" s="57"/>
       <c r="AE25" s="57"/>
       <c r="AF25" s="57"/>
@@ -11764,7 +11802,7 @@
       <c r="AI25" s="57"/>
       <c r="AJ25" s="37">
         <f t="shared" si="0"/>
-        <v>33.700000000000003</v>
+        <v>32.6</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -11782,11 +11820,11 @@
       </c>
       <c r="AO25" s="23">
         <f t="shared" si="5"/>
-        <v>32.412500000000009</v>
+        <v>32.420000000000009</v>
       </c>
       <c r="AP25" s="23">
         <f t="shared" si="4"/>
-        <v>2.0366346067789394</v>
+        <v>2.0441346067789397</v>
       </c>
     </row>
     <row r="26" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11874,7 +11912,9 @@
       <c r="AB26" s="57">
         <v>20</v>
       </c>
-      <c r="AC26" s="57"/>
+      <c r="AC26" s="57">
+        <v>19.8</v>
+      </c>
       <c r="AD26" s="57"/>
       <c r="AE26" s="57"/>
       <c r="AF26" s="57"/>
@@ -11883,7 +11923,7 @@
       <c r="AI26" s="57"/>
       <c r="AJ26" s="37">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
@@ -11901,11 +11941,11 @@
       </c>
       <c r="AO26" s="23">
         <f t="shared" si="5"/>
-        <v>19.716666666666669</v>
+        <v>19.720000000000002</v>
       </c>
       <c r="AP26" s="23">
         <f t="shared" si="4"/>
-        <v>1.1737950592233091</v>
+        <v>1.1771283925566429</v>
       </c>
     </row>
     <row r="27" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12112,7 +12152,9 @@
       <c r="AB28" s="57">
         <v>33.700000000000003</v>
       </c>
-      <c r="AC28" s="57"/>
+      <c r="AC28" s="57">
+        <v>31.4</v>
+      </c>
       <c r="AD28" s="57"/>
       <c r="AE28" s="57"/>
       <c r="AF28" s="57"/>
@@ -12121,7 +12163,7 @@
       <c r="AI28" s="57"/>
       <c r="AJ28" s="37">
         <f t="shared" si="0"/>
-        <v>33.700000000000003</v>
+        <v>31.4</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -12139,11 +12181,11 @@
       </c>
       <c r="AO28" s="23">
         <f t="shared" si="5"/>
-        <v>32.00416666666667</v>
+        <v>31.980000000000004</v>
       </c>
       <c r="AP28" s="23">
         <f t="shared" si="4"/>
-        <v>1.4757140650105107</v>
+        <v>1.4515473983438447</v>
       </c>
     </row>
     <row r="29" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12297,7 +12339,9 @@
       <c r="AB30" s="57">
         <v>37</v>
       </c>
-      <c r="AC30" s="57"/>
+      <c r="AC30" s="57">
+        <v>35.299999999999997</v>
+      </c>
       <c r="AD30" s="57"/>
       <c r="AE30" s="57"/>
       <c r="AF30" s="57"/>
@@ -12306,7 +12350,7 @@
       <c r="AI30" s="57"/>
       <c r="AJ30" s="37">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
@@ -12324,11 +12368,11 @@
       </c>
       <c r="AO30" s="23">
         <f t="shared" si="5"/>
-        <v>34.791666666666671</v>
+        <v>34.812000000000005</v>
       </c>
       <c r="AP30" s="23">
         <f t="shared" si="4"/>
-        <v>1.0494157706093219</v>
+        <v>1.0697491039426552</v>
       </c>
     </row>
     <row r="31" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12416,7 +12460,9 @@
       <c r="AB31" s="57">
         <v>26.2</v>
       </c>
-      <c r="AC31" s="57"/>
+      <c r="AC31" s="57">
+        <v>27.6</v>
+      </c>
       <c r="AD31" s="57"/>
       <c r="AE31" s="57"/>
       <c r="AF31" s="57"/>
@@ -12425,7 +12471,7 @@
       <c r="AI31" s="57"/>
       <c r="AJ31" s="37">
         <f t="shared" si="0"/>
-        <v>26.2</v>
+        <v>27.6</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
@@ -12443,11 +12489,11 @@
       </c>
       <c r="AO31" s="23">
         <f t="shared" si="5"/>
-        <v>27.237499999999997</v>
+        <v>27.251999999999999</v>
       </c>
       <c r="AP31" s="23">
         <f t="shared" si="4"/>
-        <v>1.8500751628793779</v>
+        <v>1.8645751628793796</v>
       </c>
     </row>
     <row r="32" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12535,7 +12581,9 @@
       <c r="AB32" s="57">
         <v>13</v>
       </c>
-      <c r="AC32" s="57"/>
+      <c r="AC32" s="57">
+        <v>17.399999999999999</v>
+      </c>
       <c r="AD32" s="57"/>
       <c r="AE32" s="57"/>
       <c r="AF32" s="57"/>
@@ -12544,7 +12592,7 @@
       <c r="AI32" s="57"/>
       <c r="AJ32" s="37">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="1"/>
@@ -12562,11 +12610,11 @@
       </c>
       <c r="AO32" s="23">
         <f t="shared" si="5"/>
-        <v>17.833333333333336</v>
+        <v>17.816000000000003</v>
       </c>
       <c r="AP32" s="23">
         <f t="shared" si="4"/>
-        <v>1.5037955600720849</v>
+        <v>1.4864622267387517</v>
       </c>
     </row>
     <row r="33" spans="1:47" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12654,7 +12702,9 @@
       <c r="AB33" s="57">
         <v>14.2</v>
       </c>
-      <c r="AC33" s="57"/>
+      <c r="AC33" s="57">
+        <v>15.2</v>
+      </c>
       <c r="AD33" s="57"/>
       <c r="AE33" s="57"/>
       <c r="AF33" s="57"/>
@@ -12663,7 +12713,7 @@
       <c r="AI33" s="57"/>
       <c r="AJ33" s="37">
         <f t="shared" si="0"/>
-        <v>14.2</v>
+        <v>15.2</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -12681,11 +12731,11 @@
       </c>
       <c r="AO33" s="23">
         <f t="shared" si="5"/>
-        <v>15.712499999999999</v>
+        <v>15.691999999999998</v>
       </c>
       <c r="AP33" s="23">
         <f t="shared" si="4"/>
-        <v>0.9678874675565492</v>
+        <v>0.94738746755654901</v>
       </c>
       <c r="AT33" s="15"/>
     </row>
@@ -12825,7 +12875,9 @@
       <c r="AB35" s="57">
         <v>33.200000000000003</v>
       </c>
-      <c r="AC35" s="57"/>
+      <c r="AC35" s="57">
+        <v>33.4</v>
+      </c>
       <c r="AD35" s="57"/>
       <c r="AE35" s="57"/>
       <c r="AF35" s="57"/>
@@ -12834,7 +12886,7 @@
       <c r="AI35" s="57"/>
       <c r="AJ35" s="37">
         <f t="shared" si="0"/>
-        <v>33.200000000000003</v>
+        <v>33.4</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -12852,11 +12904,11 @@
       </c>
       <c r="AO35" s="23">
         <f>IF(COUNTIF(E35:AI35,"&gt;0")&gt;=15,AVERAGE(E35:AI35),"")</f>
-        <v>31.858333333333331</v>
+        <v>31.919999999999995</v>
       </c>
       <c r="AP35" s="23">
         <f t="shared" si="4"/>
-        <v>0.78563748079876916</v>
+        <v>0.84730414746543303</v>
       </c>
       <c r="AT35" s="15"/>
     </row>
@@ -13065,7 +13117,9 @@
       <c r="AB38" s="57">
         <v>32.6</v>
       </c>
-      <c r="AC38" s="57"/>
+      <c r="AC38" s="57">
+        <v>30.7</v>
+      </c>
       <c r="AD38" s="57"/>
       <c r="AE38" s="57"/>
       <c r="AF38" s="57"/>
@@ -13074,7 +13128,7 @@
       <c r="AI38" s="57"/>
       <c r="AJ38" s="37">
         <f t="shared" si="0"/>
-        <v>32.6</v>
+        <v>30.7</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -13092,11 +13146,11 @@
       </c>
       <c r="AO38" s="23">
         <f>IF(COUNTIF(E38:AI38,"&gt;0")&gt;=15,AVERAGE(E38:AI38),"")</f>
-        <v>30.162499999999994</v>
+        <v>30.183999999999997</v>
       </c>
       <c r="AP38" s="23">
         <f t="shared" si="4"/>
-        <v>0.13347377660741344</v>
+        <v>0.15497377660741662</v>
       </c>
       <c r="AT38" s="15"/>
     </row>
@@ -13185,7 +13239,9 @@
       <c r="AB39" s="57">
         <v>32.4</v>
       </c>
-      <c r="AC39" s="57"/>
+      <c r="AC39" s="57">
+        <v>33.6</v>
+      </c>
       <c r="AD39" s="57"/>
       <c r="AE39" s="57"/>
       <c r="AF39" s="57"/>
@@ -13194,7 +13250,7 @@
       <c r="AI39" s="57"/>
       <c r="AJ39" s="37">
         <f t="shared" si="0"/>
-        <v>32.4</v>
+        <v>33.6</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
@@ -13212,11 +13268,11 @@
       </c>
       <c r="AO39" s="23">
         <f t="shared" ref="AO39:AO48" si="7">IF(COUNTIF(E39:AI39,"&gt;0")&gt;=15,AVERAGE(E39:AI39),"")</f>
-        <v>31.4375</v>
+        <v>31.524000000000001</v>
       </c>
       <c r="AP39" s="23">
         <f t="shared" si="4"/>
-        <v>0.59436688913607938</v>
+        <v>0.68086688913608029</v>
       </c>
       <c r="AT39" s="15"/>
     </row>
@@ -13305,7 +13361,9 @@
       <c r="AB40" s="57">
         <v>32.200000000000003</v>
       </c>
-      <c r="AC40" s="57"/>
+      <c r="AC40" s="57">
+        <v>31.8</v>
+      </c>
       <c r="AD40" s="57"/>
       <c r="AE40" s="57"/>
       <c r="AF40" s="57"/>
@@ -13314,7 +13372,7 @@
       <c r="AI40" s="57"/>
       <c r="AJ40" s="37">
         <f t="shared" si="0"/>
-        <v>32.200000000000003</v>
+        <v>31.8</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -13332,11 +13390,11 @@
       </c>
       <c r="AO40" s="23">
         <f t="shared" si="7"/>
-        <v>29.8125</v>
+        <v>29.891999999999999</v>
       </c>
       <c r="AP40" s="23">
         <f t="shared" si="4"/>
-        <v>0.86495161290321931</v>
+        <v>0.94445161290321877</v>
       </c>
       <c r="AT40" s="15"/>
     </row>
@@ -13425,7 +13483,9 @@
       <c r="AB41" s="57">
         <v>36</v>
       </c>
-      <c r="AC41" s="57"/>
+      <c r="AC41" s="57">
+        <v>31.4</v>
+      </c>
       <c r="AD41" s="57"/>
       <c r="AE41" s="57"/>
       <c r="AF41" s="57"/>
@@ -13434,7 +13494,7 @@
       <c r="AI41" s="57"/>
       <c r="AJ41" s="37">
         <f t="shared" si="0"/>
-        <v>36</v>
+        <v>31.4</v>
       </c>
       <c r="AK41" s="21">
         <f t="shared" si="1"/>
@@ -13452,11 +13512,11 @@
       </c>
       <c r="AO41" s="23">
         <f t="shared" si="7"/>
-        <v>30.616666666666674</v>
+        <v>30.648000000000007</v>
       </c>
       <c r="AP41" s="23">
         <f t="shared" si="4"/>
-        <v>1.2503584229390832</v>
+        <v>1.2816917562724157</v>
       </c>
       <c r="AT41" s="15"/>
     </row>
@@ -13606,7 +13666,9 @@
       <c r="AB43" s="57">
         <v>32.4</v>
       </c>
-      <c r="AC43" s="57"/>
+      <c r="AC43" s="57">
+        <v>32.6</v>
+      </c>
       <c r="AD43" s="57"/>
       <c r="AE43" s="57"/>
       <c r="AF43" s="57"/>
@@ -13615,7 +13677,7 @@
       <c r="AI43" s="57"/>
       <c r="AJ43" s="37">
         <f t="shared" si="0"/>
-        <v>32.4</v>
+        <v>32.6</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
@@ -13633,11 +13695,11 @@
       </c>
       <c r="AO43" s="23">
         <f t="shared" si="7"/>
-        <v>31.066666666666666</v>
+        <v>31.136363636363637</v>
       </c>
       <c r="AP43" s="23">
         <f t="shared" si="4"/>
-        <v>1.0056048387096759</v>
+        <v>1.0753018084066461</v>
       </c>
       <c r="AT43" s="15"/>
     </row>
@@ -13724,7 +13786,9 @@
       <c r="AB44" s="29">
         <v>32</v>
       </c>
-      <c r="AC44" s="29"/>
+      <c r="AC44" s="29">
+        <v>32</v>
+      </c>
       <c r="AD44" s="29"/>
       <c r="AE44" s="57"/>
       <c r="AF44" s="57"/>
@@ -13751,11 +13815,11 @@
       </c>
       <c r="AO44" s="23">
         <f t="shared" si="7"/>
-        <v>31.178260869565214</v>
+        <v>31.212499999999995</v>
       </c>
       <c r="AP44" s="23">
         <f t="shared" si="4"/>
-        <v>2.1350736642047536</v>
+        <v>2.1693127946395343</v>
       </c>
       <c r="AT44" s="15"/>
     </row>
@@ -13844,7 +13908,9 @@
       <c r="AB45" s="57">
         <v>33.6</v>
       </c>
-      <c r="AC45" s="57"/>
+      <c r="AC45" s="57">
+        <v>33.200000000000003</v>
+      </c>
       <c r="AD45" s="57"/>
       <c r="AE45" s="57"/>
       <c r="AF45" s="57"/>
@@ -13853,7 +13919,7 @@
       <c r="AI45" s="57"/>
       <c r="AJ45" s="37">
         <f t="shared" si="0"/>
-        <v>33.6</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -13871,11 +13937,11 @@
       </c>
       <c r="AO45" s="23">
         <f t="shared" si="7"/>
-        <v>30.516666666666676</v>
+        <v>30.624000000000009</v>
       </c>
       <c r="AP45" s="23">
         <f t="shared" si="4"/>
-        <v>0.97085027378784616</v>
+        <v>1.0781836071211792</v>
       </c>
       <c r="AT45" s="15"/>
     </row>
@@ -14103,7 +14169,9 @@
       <c r="AB48" s="57">
         <v>29</v>
       </c>
-      <c r="AC48" s="57"/>
+      <c r="AC48" s="57">
+        <v>30.2</v>
+      </c>
       <c r="AD48" s="57"/>
       <c r="AE48" s="57"/>
       <c r="AF48" s="57"/>
@@ -14112,7 +14180,7 @@
       <c r="AI48" s="57"/>
       <c r="AJ48" s="37">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>30.2</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="1"/>
@@ -14130,11 +14198,11 @@
       </c>
       <c r="AO48" s="23">
         <f t="shared" si="7"/>
-        <v>30.729166666666668</v>
+        <v>30.708000000000002</v>
       </c>
       <c r="AP48" s="23">
         <f t="shared" si="4"/>
-        <v>0.38663381123058826</v>
+        <v>0.36546714456392237</v>
       </c>
     </row>
     <row r="49" spans="5:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -27033,12 +27101,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -27048,6 +27110,12 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>